<commit_message>
WORKING.  specify format for course lookup
</commit_message>
<xml_diff>
--- a/cloudapp/src/assets/example input.xlsx
+++ b/cloudapp/src/assets/example input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\WebRoot\hsteele\mms_lookup_v9_backup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hsteel01\Desktop\item-updater-excel\tufts-alma-cloudapp-citation-loader-v2\cloudapp\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCBBBED6-03A6-4A82-A8D3-31F06138A73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA255D0D-6F1D-4290-BB05-62A9B215248D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A7A01D49-2CA6-49F1-9BC2-FD03B27F406D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
   <si>
     <t>Title</t>
   </si>
@@ -141,6 +141,18 @@
   </si>
   <si>
     <t>Contributor First</t>
+  </si>
+  <si>
+    <t>Course Year for Mapping</t>
+  </si>
+  <si>
+    <t>Course Term for Mapping</t>
+  </si>
+  <si>
+    <t>02  or something else, or  blank if you use the Course Semester column</t>
+  </si>
+  <si>
+    <t>2024 or blank if using Course Semester Field</t>
   </si>
 </sst>
 </file>
@@ -562,10 +574,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57814615-5594-4B02-B3B4-74560264A7D8}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -597,13 +609,19 @@
         <v>15</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="52.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>28</v>
       </c>
@@ -628,11 +646,17 @@
       <c r="J2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="84" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="84" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>30</v>
       </c>
@@ -659,14 +683,20 @@
       <c r="J3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" t="s">
         <v>18</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="73.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="73.5" x14ac:dyDescent="0.45">
       <c r="A4" s="3"/>
       <c r="C4" t="s">
         <v>26</v>
@@ -692,14 +722,20 @@
       <c r="J4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" t="s">
         <v>19</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="84" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="84" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -726,14 +762,20 @@
       <c r="J5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" t="s">
         <v>20</v>
       </c>
-      <c r="L5" t="s">
+      <c r="N5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="16" x14ac:dyDescent="0.45">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -744,6 +786,8 @@
       <c r="H6" s="4"/>
       <c r="I6" s="5"/>
       <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>